<commit_message>
PLAN-013a Batch B: the owner's business data out of the repository (B1–B2). docs/inputs/ (nine files) removed and its README says where they live (the private container owner-inputs, the owner's account alone); the store-cost templates replaced by invented rows (the real rows moved out with the inputs); real store numbers with towns, the revenue total and the staff names redacted to placeholders in SCOPE, COLUMN_MAPPING and STATUS; the test data's real towns and the August fixture's real total replaced by invented ones (the example and fixture spreadsheets regenerated). History is not rewritten.
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/store_costs/two_rows.xlsx
+++ b/backend/tests/fixtures/store_costs/two_rows.xlsx
@@ -17,9 +17,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -50,10 +49,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -487,7 +487,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AMHERST, NH</t>
+          <t>Town A, NH</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -498,10 +498,10 @@
       <c r="F2" s="1" t="n">
         <v>2500</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="3" t="n">
         <v>46023</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="3" t="n">
         <v>47848</v>
       </c>
       <c r="I2" s="1" t="n"/>
@@ -514,7 +514,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SEALY, TEXAS</t>
+          <t>Town B, TX</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,10 +525,10 @@
       <c r="F3" s="1" t="n">
         <v>3000</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="3" t="n">
         <v>46023</v>
       </c>
-      <c r="H3" s="2" t="n"/>
+      <c r="H3" s="3" t="n"/>
       <c r="I3" s="1" t="n">
         <v>50</v>
       </c>

</xml_diff>